<commit_message>
did more to_excel and pfd functions, created cooling tower station and juice heating station. updated main
</commit_message>
<xml_diff>
--- a/four_boiling.xlsx
+++ b/four_boiling.xlsx
@@ -588,10 +588,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I261"/>
+  <dimension ref="A1:I262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -5613,6 +5613,14 @@
           <t>°F</t>
         </is>
       </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="17" t="inlineStr">
+        <is>
+          <t>Note: if using CoolingTowerSystem, ignore these injection water demands - they are re-solved there at the delivered water temp.</t>
+        </is>
+      </c>
+      <c r="B262" s="20" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="21">

</xml_diff>